<commit_message>
fix: deterministic short_kernels_summary sort and address Copilot review
Add string-typed groupby columns as tie-breakers to short_kernels_summary
sort so rows with the same duration sum have reproducible ordering.
Regenerate all reference xlsx files. Fix tmpdir leak in jax perf report
test, clarify protobuf pin comment, and update README sidecar description.
</commit_message>
<xml_diff>
--- a/tests/traces/compare_test_e2e/reference/h100_perf_report.xlsx
+++ b/tests/traces/compare_test_e2e/reference/h100_perf_report.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SDPA_fwd" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Reduce_fwd" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="kernel_summary" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="short_kernel_histogram" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="short_kernels_summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gpu_timeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary_by_category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ops_unique_args" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unified_perf_summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEMM" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDPA_fwd" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BinaryElementwise" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UnaryElementwise" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduce_fwd" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kernel_summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="short_kernel_histogram" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="short_kernels_summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>